<commit_message>
Add Budget vs. Actual page to Finance section
</commit_message>
<xml_diff>
--- a/Fire Department 2026 Git/Fire Data/ElCerrito_GF_Budget_vs_Actual_FY14-FY25.xlsx
+++ b/Fire Department 2026 Git/Fire Data/ElCerrito_GF_Budget_vs_Actual_FY14-FY25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Employment\2026 job search\GitHub\portfolio\Fire Department 2026 Git\Fire Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{0BAD446D-AB7A-433A-9BEF-EAD1903D8B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7647D27-B345-4C54-9CCB-AD957E6DC1F2}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{0BAD446D-AB7A-433A-9BEF-EAD1903D8B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA54172D-2CDE-476D-B4E7-FCED7134B3E7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="79">
   <si>
     <t>City of El Cerrito — General Fund Budget vs. Actual, FY 2013-14 through FY 2024-25</t>
   </si>
@@ -279,6 +279,9 @@
   </si>
   <si>
     <t>Actual Exp - Actual Rev</t>
+  </si>
+  <si>
+    <t>Omit 20-24</t>
   </si>
 </sst>
 </file>
@@ -383,7 +386,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -415,6 +418,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -710,7 +714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{238399B8-7AF7-4C5A-B206-9E0C35CEBB08}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -1264,6 +1268,35 @@
       <c r="G17" s="8">
         <f t="shared" si="3"/>
         <v>460268118</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="14">
+        <f>SUM(B5:B10,B16)</f>
+        <v>244780343</v>
+      </c>
+      <c r="C19" s="14">
+        <f t="shared" ref="C19:G19" si="4">SUM(C5:C10,C16)</f>
+        <v>247932063</v>
+      </c>
+      <c r="D19" s="14">
+        <f t="shared" si="4"/>
+        <v>252575406</v>
+      </c>
+      <c r="E19" s="14">
+        <f t="shared" si="4"/>
+        <v>242695318</v>
+      </c>
+      <c r="F19" s="14">
+        <f t="shared" si="4"/>
+        <v>246274800</v>
+      </c>
+      <c r="G19" s="14">
+        <f t="shared" si="4"/>
+        <v>251025820</v>
       </c>
     </row>
   </sheetData>

</xml_diff>